<commit_message>
new .ttl from Google sheet has been generated
</commit_message>
<xml_diff>
--- a/elter_cl.xlsx
+++ b/elter_cl.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE676"/>
+  <dimension ref="A1:BE692"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>11/6/2025</t>
+          <t>11/26/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -50742,7 +50742,11 @@
           <t>Marine habitats</t>
         </is>
       </c>
-      <c r="C574" t="inlineStr"/>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D574" t="inlineStr">
         <is>
           <t>https://w3id.org/np/RAkLyP_I8O3ocqgRKBTmPQhedjs9KWedeEK0YdT9yfTWA#EunisHabitat,skos:Concept</t>
@@ -50787,7 +50791,7 @@
       <c r="AK574" t="inlineStr"/>
       <c r="AL574" t="inlineStr">
         <is>
-          <t>0000-0003-2195-3997</t>
+          <t>0000-0003-2195-3997, 0000-0002-7997-219X</t>
         </is>
       </c>
       <c r="AM574" t="inlineStr">
@@ -50798,7 +50802,7 @@
       <c r="AN574" t="inlineStr"/>
       <c r="AO574" t="inlineStr">
         <is>
-          <t>6/26/2024</t>
+          <t>11/26/2025</t>
         </is>
       </c>
       <c r="AP574" t="inlineStr"/>
@@ -50829,7 +50833,11 @@
           <t>Inland surface waters</t>
         </is>
       </c>
-      <c r="C575" t="inlineStr"/>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="D575" t="inlineStr">
         <is>
           <t>https://w3id.org/np/RAkLyP_I8O3ocqgRKBTmPQhedjs9KWedeEK0YdT9yfTWA#EunisHabitat,skos:Concept</t>
@@ -50885,7 +50893,7 @@
       <c r="AN575" t="inlineStr"/>
       <c r="AO575" t="inlineStr">
         <is>
-          <t>6/26/2024</t>
+          <t>11/26/2025</t>
         </is>
       </c>
       <c r="AP575" t="inlineStr"/>
@@ -50916,7 +50924,11 @@
           <t>Mires, bogs and fens</t>
         </is>
       </c>
-      <c r="C576" t="inlineStr"/>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="D576" t="inlineStr">
         <is>
           <t>https://w3id.org/np/RAkLyP_I8O3ocqgRKBTmPQhedjs9KWedeEK0YdT9yfTWA#EunisHabitat,skos:Concept</t>
@@ -50972,7 +50984,7 @@
       <c r="AN576" t="inlineStr"/>
       <c r="AO576" t="inlineStr">
         <is>
-          <t>6/26/2024</t>
+          <t>11/26/2025</t>
         </is>
       </c>
       <c r="AP576" t="inlineStr"/>
@@ -51003,7 +51015,11 @@
           <t>Grasslands and lands dominated by forbs, mosses or lichens</t>
         </is>
       </c>
-      <c r="C577" t="inlineStr"/>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="D577" t="inlineStr">
         <is>
           <t>https://w3id.org/np/RAkLyP_I8O3ocqgRKBTmPQhedjs9KWedeEK0YdT9yfTWA#EunisHabitat,skos:Concept</t>
@@ -51059,7 +51075,7 @@
       <c r="AN577" t="inlineStr"/>
       <c r="AO577" t="inlineStr">
         <is>
-          <t>6/26/2024</t>
+          <t>11/26/2025</t>
         </is>
       </c>
       <c r="AP577" t="inlineStr"/>
@@ -51090,7 +51106,11 @@
           <t>Heathlands, scrub and tundra</t>
         </is>
       </c>
-      <c r="C578" t="inlineStr"/>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
       <c r="D578" t="inlineStr">
         <is>
           <t>https://w3id.org/np/RAkLyP_I8O3ocqgRKBTmPQhedjs9KWedeEK0YdT9yfTWA#EunisHabitat,skos:Concept</t>
@@ -51146,7 +51166,7 @@
       <c r="AN578" t="inlineStr"/>
       <c r="AO578" t="inlineStr">
         <is>
-          <t>6/26/2024</t>
+          <t>11/26/2025</t>
         </is>
       </c>
       <c r="AP578" t="inlineStr"/>
@@ -51177,7 +51197,11 @@
           <t>Woodland, forest and other wooded land</t>
         </is>
       </c>
-      <c r="C579" t="inlineStr"/>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
       <c r="D579" t="inlineStr">
         <is>
           <t>https://w3id.org/np/RAkLyP_I8O3ocqgRKBTmPQhedjs9KWedeEK0YdT9yfTWA#EunisHabitat,skos:Concept</t>
@@ -51233,7 +51257,7 @@
       <c r="AN579" t="inlineStr"/>
       <c r="AO579" t="inlineStr">
         <is>
-          <t>6/26/2024</t>
+          <t>11/26/2025</t>
         </is>
       </c>
       <c r="AP579" t="inlineStr"/>
@@ -51264,7 +51288,11 @@
           <t>Inland unvegetated or sparsely vegetated habitats</t>
         </is>
       </c>
-      <c r="C580" t="inlineStr"/>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
       <c r="D580" t="inlineStr">
         <is>
           <t>https://w3id.org/np/RAkLyP_I8O3ocqgRKBTmPQhedjs9KWedeEK0YdT9yfTWA#EunisHabitat,skos:Concept</t>
@@ -51320,7 +51348,7 @@
       <c r="AN580" t="inlineStr"/>
       <c r="AO580" t="inlineStr">
         <is>
-          <t>6/26/2024</t>
+          <t>11/26/2025</t>
         </is>
       </c>
       <c r="AP580" t="inlineStr"/>
@@ -51351,7 +51379,11 @@
           <t>Regularly or recently cultivated agricultural, horticultural and domestic habitats</t>
         </is>
       </c>
-      <c r="C581" t="inlineStr"/>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="D581" t="inlineStr">
         <is>
           <t>https://w3id.org/np/RAkLyP_I8O3ocqgRKBTmPQhedjs9KWedeEK0YdT9yfTWA#EunisHabitat,skos:Concept</t>
@@ -51407,7 +51439,7 @@
       <c r="AN581" t="inlineStr"/>
       <c r="AO581" t="inlineStr">
         <is>
-          <t>6/26/2024</t>
+          <t>11/26/2025</t>
         </is>
       </c>
       <c r="AP581" t="inlineStr"/>
@@ -54223,7 +54255,11 @@
         </is>
       </c>
       <c r="C614" t="inlineStr"/>
-      <c r="D614" t="inlineStr"/>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>https://w3id.org/np/RAkLyP_I8O3ocqgRKBTmPQhedjs9KWedeEK0YdT9yfTWA#EunisHabitat,skos:Concept</t>
+        </is>
+      </c>
       <c r="E614" t="inlineStr"/>
       <c r="F614" t="inlineStr"/>
       <c r="G614" t="inlineStr"/>
@@ -54278,7 +54314,7 @@
       </c>
       <c r="AO614" t="inlineStr">
         <is>
-          <t>10/16/2023</t>
+          <t>11/26/2025</t>
         </is>
       </c>
       <c r="AP614" t="inlineStr"/>
@@ -54396,7 +54432,11 @@
           <t>Coastal habitats</t>
         </is>
       </c>
-      <c r="C616" t="inlineStr"/>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="D616" t="inlineStr">
         <is>
           <t>https://w3id.org/np/RAkLyP_I8O3ocqgRKBTmPQhedjs9KWedeEK0YdT9yfTWA#EunisHabitat,skos:Concept</t>
@@ -54456,7 +54496,7 @@
       </c>
       <c r="AO616" t="inlineStr">
         <is>
-          <t>6/26/2024</t>
+          <t>11/26/2025</t>
         </is>
       </c>
       <c r="AP616" t="inlineStr"/>
@@ -59810,10 +59850,14 @@
           <t>6/28/2024</t>
         </is>
       </c>
-      <c r="AN676" t="inlineStr"/>
+      <c r="AN676" t="inlineStr">
+        <is>
+          <t>0000-0003-2195-3997</t>
+        </is>
+      </c>
       <c r="AO676" t="inlineStr">
         <is>
-          <t>8/27/2024</t>
+          <t>11/26/2025</t>
         </is>
       </c>
       <c r="AP676" t="inlineStr"/>
@@ -59833,6 +59877,1522 @@
       <c r="BD676" t="inlineStr"/>
       <c r="BE676" t="inlineStr"/>
     </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>cl:10754</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Data Level</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>data level, eLTER data level</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr"/>
+      <c r="F677" t="inlineStr"/>
+      <c r="G677" t="inlineStr"/>
+      <c r="H677" t="inlineStr"/>
+      <c r="I677" t="inlineStr"/>
+      <c r="J677" t="inlineStr"/>
+      <c r="K677" t="inlineStr"/>
+      <c r="L677" t="inlineStr"/>
+      <c r="M677" t="inlineStr"/>
+      <c r="N677" t="inlineStr"/>
+      <c r="O677" t="inlineStr"/>
+      <c r="P677" t="inlineStr"/>
+      <c r="Q677" t="inlineStr"/>
+      <c r="R677" t="inlineStr"/>
+      <c r="S677" t="inlineStr"/>
+      <c r="T677" t="inlineStr"/>
+      <c r="U677" t="inlineStr"/>
+      <c r="V677" t="inlineStr"/>
+      <c r="W677" t="inlineStr"/>
+      <c r="X677" t="inlineStr"/>
+      <c r="Y677" t="inlineStr"/>
+      <c r="Z677" t="inlineStr"/>
+      <c r="AA677" t="inlineStr"/>
+      <c r="AB677" t="inlineStr"/>
+      <c r="AC677" t="inlineStr"/>
+      <c r="AD677" t="inlineStr"/>
+      <c r="AE677" t="inlineStr"/>
+      <c r="AF677" t="inlineStr"/>
+      <c r="AG677" t="inlineStr"/>
+      <c r="AH677" t="inlineStr"/>
+      <c r="AI677" t="inlineStr"/>
+      <c r="AJ677" t="inlineStr"/>
+      <c r="AK677" t="inlineStr"/>
+      <c r="AL677" t="inlineStr"/>
+      <c r="AM677" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN677" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO677" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP677" t="inlineStr"/>
+      <c r="AQ677" t="inlineStr"/>
+      <c r="AR677" t="inlineStr"/>
+      <c r="AS677" t="inlineStr"/>
+      <c r="AT677" t="inlineStr"/>
+      <c r="AU677" t="inlineStr"/>
+      <c r="AV677" t="inlineStr"/>
+      <c r="AW677" t="inlineStr"/>
+      <c r="AX677" t="inlineStr"/>
+      <c r="AY677" t="inlineStr"/>
+      <c r="AZ677" t="inlineStr"/>
+      <c r="BA677" t="inlineStr"/>
+      <c r="BB677" t="inlineStr"/>
+      <c r="BC677" t="inlineStr"/>
+      <c r="BD677" t="inlineStr"/>
+      <c r="BE677" t="inlineStr"/>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>cl:10755</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Raw data</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>0, Level 0</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr"/>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>Are defined as Raw data, which are values directly obtained by human measurements or automated sensors that have not undergone any transformation. This could include quantitative or qualitative information about physical variables of the environment and may be of various forms, such as images, text files or physical samples. These data are transformed into physical units either directly provided by instruments or converted from engineering units (for example, mV, mA, Ω) to physical units.</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr"/>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>cl:10754</t>
+        </is>
+      </c>
+      <c r="I678" t="inlineStr"/>
+      <c r="J678" t="inlineStr"/>
+      <c r="K678" t="inlineStr"/>
+      <c r="L678" t="inlineStr"/>
+      <c r="M678" t="inlineStr"/>
+      <c r="N678" t="inlineStr"/>
+      <c r="O678" t="inlineStr"/>
+      <c r="P678" t="inlineStr"/>
+      <c r="Q678" t="inlineStr"/>
+      <c r="R678" t="inlineStr"/>
+      <c r="S678" t="inlineStr"/>
+      <c r="T678" t="inlineStr"/>
+      <c r="U678" t="inlineStr"/>
+      <c r="V678" t="inlineStr"/>
+      <c r="W678" t="inlineStr"/>
+      <c r="X678" t="inlineStr"/>
+      <c r="Y678" t="inlineStr"/>
+      <c r="Z678" t="inlineStr"/>
+      <c r="AA678" t="inlineStr"/>
+      <c r="AB678" t="inlineStr">
+        <is>
+          <t>Raw data in physical units directly from a sensor with original temporal and spatial resolution.</t>
+        </is>
+      </c>
+      <c r="AC678" t="inlineStr"/>
+      <c r="AD678" t="inlineStr"/>
+      <c r="AE678" t="inlineStr"/>
+      <c r="AF678" t="inlineStr"/>
+      <c r="AG678" t="inlineStr"/>
+      <c r="AH678" t="inlineStr"/>
+      <c r="AI678" t="inlineStr"/>
+      <c r="AJ678" t="inlineStr"/>
+      <c r="AK678" t="inlineStr"/>
+      <c r="AL678" t="inlineStr"/>
+      <c r="AM678" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN678" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO678" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP678" t="inlineStr"/>
+      <c r="AQ678" t="inlineStr"/>
+      <c r="AR678" t="inlineStr"/>
+      <c r="AS678" t="inlineStr"/>
+      <c r="AT678" t="inlineStr"/>
+      <c r="AU678" t="inlineStr"/>
+      <c r="AV678" t="inlineStr"/>
+      <c r="AW678" t="inlineStr"/>
+      <c r="AX678" t="inlineStr"/>
+      <c r="AY678" t="inlineStr"/>
+      <c r="AZ678" t="inlineStr"/>
+      <c r="BA678" t="inlineStr"/>
+      <c r="BB678" t="inlineStr"/>
+      <c r="BC678" t="inlineStr"/>
+      <c r="BD678" t="inlineStr"/>
+      <c r="BE678" t="inlineStr"/>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>cl:10756</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Observation data</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>1, Level 1</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr"/>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>Are defined as Observation data, which are unprocessed and have not undergone any refinement or only basic data quality control. Possible sub levels in the eLTER workflows (still need to be discussed): L1a first level of quality control by the data provider, L1b second level of quality control by central eLTER processes and centrally approved.</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr"/>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>cl:10754</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr"/>
+      <c r="J679" t="inlineStr"/>
+      <c r="K679" t="inlineStr"/>
+      <c r="L679" t="inlineStr"/>
+      <c r="M679" t="inlineStr"/>
+      <c r="N679" t="inlineStr"/>
+      <c r="O679" t="inlineStr"/>
+      <c r="P679" t="inlineStr"/>
+      <c r="Q679" t="inlineStr"/>
+      <c r="R679" t="inlineStr"/>
+      <c r="S679" t="inlineStr"/>
+      <c r="T679" t="inlineStr"/>
+      <c r="U679" t="inlineStr"/>
+      <c r="V679" t="inlineStr"/>
+      <c r="W679" t="inlineStr"/>
+      <c r="X679" t="inlineStr"/>
+      <c r="Y679" t="inlineStr"/>
+      <c r="Z679" t="inlineStr"/>
+      <c r="AA679" t="inlineStr"/>
+      <c r="AB679" t="inlineStr">
+        <is>
+          <t>Transformed and quality controlled data with original temporal and spatial resolution.</t>
+        </is>
+      </c>
+      <c r="AC679" t="inlineStr"/>
+      <c r="AD679" t="inlineStr"/>
+      <c r="AE679" t="inlineStr"/>
+      <c r="AF679" t="inlineStr"/>
+      <c r="AG679" t="inlineStr"/>
+      <c r="AH679" t="inlineStr"/>
+      <c r="AI679" t="inlineStr"/>
+      <c r="AJ679" t="inlineStr"/>
+      <c r="AK679" t="inlineStr"/>
+      <c r="AL679" t="inlineStr"/>
+      <c r="AM679" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN679" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO679" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP679" t="inlineStr"/>
+      <c r="AQ679" t="inlineStr"/>
+      <c r="AR679" t="inlineStr"/>
+      <c r="AS679" t="inlineStr"/>
+      <c r="AT679" t="inlineStr"/>
+      <c r="AU679" t="inlineStr"/>
+      <c r="AV679" t="inlineStr"/>
+      <c r="AW679" t="inlineStr"/>
+      <c r="AX679" t="inlineStr"/>
+      <c r="AY679" t="inlineStr"/>
+      <c r="AZ679" t="inlineStr"/>
+      <c r="BA679" t="inlineStr"/>
+      <c r="BB679" t="inlineStr"/>
+      <c r="BC679" t="inlineStr"/>
+      <c r="BD679" t="inlineStr"/>
+      <c r="BE679" t="inlineStr"/>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>cl:10757</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Cleaned data</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>2, Level 2</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr"/>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>Are defined as Cleaned data, which were subject to quality control procedures (either automatic and/or manual). These data passed the quality control procedures such as routine estimation of timing and sensor calibration and/or statistical/visual inspection to identify outliers and errors in the data. This can also include gap filling of missing data. Level 2 are therefore Cleaned Data that are the final, quality-checked and gap-filled, and published by the local nodes or the central data node (CDN).</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr"/>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>cl:10754</t>
+        </is>
+      </c>
+      <c r="I680" t="inlineStr"/>
+      <c r="J680" t="inlineStr"/>
+      <c r="K680" t="inlineStr"/>
+      <c r="L680" t="inlineStr"/>
+      <c r="M680" t="inlineStr"/>
+      <c r="N680" t="inlineStr"/>
+      <c r="O680" t="inlineStr"/>
+      <c r="P680" t="inlineStr"/>
+      <c r="Q680" t="inlineStr"/>
+      <c r="R680" t="inlineStr"/>
+      <c r="S680" t="inlineStr"/>
+      <c r="T680" t="inlineStr"/>
+      <c r="U680" t="inlineStr"/>
+      <c r="V680" t="inlineStr"/>
+      <c r="W680" t="inlineStr"/>
+      <c r="X680" t="inlineStr"/>
+      <c r="Y680" t="inlineStr"/>
+      <c r="Z680" t="inlineStr"/>
+      <c r="AA680" t="inlineStr"/>
+      <c r="AB680" t="inlineStr">
+        <is>
+          <t>Gap filled data with orginal temporal and spatial resolution.</t>
+        </is>
+      </c>
+      <c r="AC680" t="inlineStr"/>
+      <c r="AD680" t="inlineStr"/>
+      <c r="AE680" t="inlineStr"/>
+      <c r="AF680" t="inlineStr"/>
+      <c r="AG680" t="inlineStr"/>
+      <c r="AH680" t="inlineStr"/>
+      <c r="AI680" t="inlineStr"/>
+      <c r="AJ680" t="inlineStr"/>
+      <c r="AK680" t="inlineStr"/>
+      <c r="AL680" t="inlineStr"/>
+      <c r="AM680" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN680" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO680" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP680" t="inlineStr"/>
+      <c r="AQ680" t="inlineStr"/>
+      <c r="AR680" t="inlineStr"/>
+      <c r="AS680" t="inlineStr"/>
+      <c r="AT680" t="inlineStr"/>
+      <c r="AU680" t="inlineStr"/>
+      <c r="AV680" t="inlineStr"/>
+      <c r="AW680" t="inlineStr"/>
+      <c r="AX680" t="inlineStr"/>
+      <c r="AY680" t="inlineStr"/>
+      <c r="AZ680" t="inlineStr"/>
+      <c r="BA680" t="inlineStr"/>
+      <c r="BB680" t="inlineStr"/>
+      <c r="BC680" t="inlineStr"/>
+      <c r="BD680" t="inlineStr"/>
+      <c r="BE680" t="inlineStr"/>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>cl:10758</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Derived data</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>3, Level 3</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr"/>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>Are defined as Data Products, which are derived from quality-controlled data. They require scientific and technical interpretation and may include multi-sensor data, analytical workflows and interpretations, model-based interpretation using also other data to generate the data products. Data products reflect a diversity of products elaborated by scientific communities that rely partly or completely on eLTER lower-level data. eLTER will provide resources to integrate and disseminate Level 3 products.</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr"/>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>cl:10754</t>
+        </is>
+      </c>
+      <c r="I681" t="inlineStr"/>
+      <c r="J681" t="inlineStr"/>
+      <c r="K681" t="inlineStr"/>
+      <c r="L681" t="inlineStr"/>
+      <c r="M681" t="inlineStr"/>
+      <c r="N681" t="inlineStr"/>
+      <c r="O681" t="inlineStr"/>
+      <c r="P681" t="inlineStr"/>
+      <c r="Q681" t="inlineStr"/>
+      <c r="R681" t="inlineStr"/>
+      <c r="S681" t="inlineStr"/>
+      <c r="T681" t="inlineStr"/>
+      <c r="U681" t="inlineStr"/>
+      <c r="V681" t="inlineStr"/>
+      <c r="W681" t="inlineStr"/>
+      <c r="X681" t="inlineStr"/>
+      <c r="Y681" t="inlineStr"/>
+      <c r="Z681" t="inlineStr"/>
+      <c r="AA681" t="inlineStr"/>
+      <c r="AB681" t="inlineStr">
+        <is>
+          <t>Modelled data or aggregated data (e.g. monthly aggregation harmonised across eLTER facilities).</t>
+        </is>
+      </c>
+      <c r="AC681" t="inlineStr"/>
+      <c r="AD681" t="inlineStr"/>
+      <c r="AE681" t="inlineStr"/>
+      <c r="AF681" t="inlineStr"/>
+      <c r="AG681" t="inlineStr"/>
+      <c r="AH681" t="inlineStr"/>
+      <c r="AI681" t="inlineStr"/>
+      <c r="AJ681" t="inlineStr"/>
+      <c r="AK681" t="inlineStr"/>
+      <c r="AL681" t="inlineStr"/>
+      <c r="AM681" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN681" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO681" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP681" t="inlineStr"/>
+      <c r="AQ681" t="inlineStr"/>
+      <c r="AR681" t="inlineStr"/>
+      <c r="AS681" t="inlineStr"/>
+      <c r="AT681" t="inlineStr"/>
+      <c r="AU681" t="inlineStr"/>
+      <c r="AV681" t="inlineStr"/>
+      <c r="AW681" t="inlineStr"/>
+      <c r="AX681" t="inlineStr"/>
+      <c r="AY681" t="inlineStr"/>
+      <c r="AZ681" t="inlineStr"/>
+      <c r="BA681" t="inlineStr"/>
+      <c r="BB681" t="inlineStr"/>
+      <c r="BC681" t="inlineStr"/>
+      <c r="BD681" t="inlineStr"/>
+      <c r="BE681" t="inlineStr"/>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>cl:10759</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>SO habitats</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr"/>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr"/>
+      <c r="F682" t="inlineStr"/>
+      <c r="G682" t="inlineStr"/>
+      <c r="H682" t="inlineStr"/>
+      <c r="I682" t="inlineStr"/>
+      <c r="J682" t="inlineStr"/>
+      <c r="K682" t="inlineStr"/>
+      <c r="L682" t="inlineStr"/>
+      <c r="M682" t="inlineStr"/>
+      <c r="N682" t="inlineStr"/>
+      <c r="O682" t="inlineStr"/>
+      <c r="P682" t="inlineStr"/>
+      <c r="Q682" t="inlineStr"/>
+      <c r="R682" t="inlineStr"/>
+      <c r="S682" t="inlineStr"/>
+      <c r="T682" t="inlineStr"/>
+      <c r="U682" t="inlineStr"/>
+      <c r="V682" t="inlineStr"/>
+      <c r="W682" t="inlineStr"/>
+      <c r="X682" t="inlineStr"/>
+      <c r="Y682" t="inlineStr"/>
+      <c r="Z682" t="inlineStr"/>
+      <c r="AA682" t="inlineStr"/>
+      <c r="AB682" t="inlineStr"/>
+      <c r="AC682" t="inlineStr"/>
+      <c r="AD682" t="inlineStr"/>
+      <c r="AE682" t="inlineStr"/>
+      <c r="AF682" t="inlineStr"/>
+      <c r="AG682" t="inlineStr"/>
+      <c r="AH682" t="inlineStr"/>
+      <c r="AI682" t="inlineStr"/>
+      <c r="AJ682" t="inlineStr"/>
+      <c r="AK682" t="inlineStr"/>
+      <c r="AL682" t="inlineStr"/>
+      <c r="AM682" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN682" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO682" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP682" t="inlineStr"/>
+      <c r="AQ682" t="inlineStr"/>
+      <c r="AR682" t="inlineStr"/>
+      <c r="AS682" t="inlineStr"/>
+      <c r="AT682" t="inlineStr"/>
+      <c r="AU682" t="inlineStr"/>
+      <c r="AV682" t="inlineStr"/>
+      <c r="AW682" t="inlineStr"/>
+      <c r="AX682" t="inlineStr"/>
+      <c r="AY682" t="inlineStr"/>
+      <c r="AZ682" t="inlineStr"/>
+      <c r="BA682" t="inlineStr"/>
+      <c r="BB682" t="inlineStr"/>
+      <c r="BC682" t="inlineStr"/>
+      <c r="BD682" t="inlineStr"/>
+      <c r="BE682" t="inlineStr"/>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>cl:10760</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Marine habitats</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr"/>
+      <c r="F683" t="inlineStr"/>
+      <c r="G683" t="inlineStr"/>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>cl:10759</t>
+        </is>
+      </c>
+      <c r="I683" t="inlineStr"/>
+      <c r="J683" t="inlineStr"/>
+      <c r="K683" t="inlineStr"/>
+      <c r="L683" t="inlineStr"/>
+      <c r="M683" t="inlineStr"/>
+      <c r="N683" t="inlineStr"/>
+      <c r="O683" t="inlineStr"/>
+      <c r="P683" t="inlineStr"/>
+      <c r="Q683" t="inlineStr"/>
+      <c r="R683" t="inlineStr"/>
+      <c r="S683" t="inlineStr"/>
+      <c r="T683" t="inlineStr"/>
+      <c r="U683" t="inlineStr"/>
+      <c r="V683" t="inlineStr"/>
+      <c r="W683" t="inlineStr"/>
+      <c r="X683" t="inlineStr"/>
+      <c r="Y683" t="inlineStr"/>
+      <c r="Z683" t="inlineStr"/>
+      <c r="AA683" t="inlineStr"/>
+      <c r="AB683" t="inlineStr"/>
+      <c r="AC683" t="inlineStr"/>
+      <c r="AD683" t="inlineStr"/>
+      <c r="AE683" t="inlineStr"/>
+      <c r="AF683" t="inlineStr"/>
+      <c r="AG683" t="inlineStr"/>
+      <c r="AH683" t="inlineStr"/>
+      <c r="AI683" t="inlineStr"/>
+      <c r="AJ683" t="inlineStr">
+        <is>
+          <t>cl:10649</t>
+        </is>
+      </c>
+      <c r="AK683" t="inlineStr"/>
+      <c r="AL683" t="inlineStr"/>
+      <c r="AM683" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN683" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO683" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP683" t="inlineStr"/>
+      <c r="AQ683" t="inlineStr"/>
+      <c r="AR683" t="inlineStr"/>
+      <c r="AS683" t="inlineStr"/>
+      <c r="AT683" t="inlineStr"/>
+      <c r="AU683" t="inlineStr"/>
+      <c r="AV683" t="inlineStr"/>
+      <c r="AW683" t="inlineStr"/>
+      <c r="AX683" t="inlineStr"/>
+      <c r="AY683" t="inlineStr"/>
+      <c r="AZ683" t="inlineStr"/>
+      <c r="BA683" t="inlineStr"/>
+      <c r="BB683" t="inlineStr"/>
+      <c r="BC683" t="inlineStr"/>
+      <c r="BD683" t="inlineStr"/>
+      <c r="BE683" t="inlineStr"/>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>cl:10761</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Coastal (transitional) waters including coastal littoral zones</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr"/>
+      <c r="F684" t="inlineStr"/>
+      <c r="G684" t="inlineStr"/>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>cl:10759</t>
+        </is>
+      </c>
+      <c r="I684" t="inlineStr"/>
+      <c r="J684" t="inlineStr"/>
+      <c r="K684" t="inlineStr"/>
+      <c r="L684" t="inlineStr"/>
+      <c r="M684" t="inlineStr"/>
+      <c r="N684" t="inlineStr"/>
+      <c r="O684" t="inlineStr"/>
+      <c r="P684" t="inlineStr"/>
+      <c r="Q684" t="inlineStr"/>
+      <c r="R684" t="inlineStr"/>
+      <c r="S684" t="inlineStr"/>
+      <c r="T684" t="inlineStr"/>
+      <c r="U684" t="inlineStr"/>
+      <c r="V684" t="inlineStr"/>
+      <c r="W684" t="inlineStr"/>
+      <c r="X684" t="inlineStr"/>
+      <c r="Y684" t="inlineStr"/>
+      <c r="Z684" t="inlineStr"/>
+      <c r="AA684" t="inlineStr"/>
+      <c r="AB684" t="inlineStr"/>
+      <c r="AC684" t="inlineStr"/>
+      <c r="AD684" t="inlineStr"/>
+      <c r="AE684" t="inlineStr"/>
+      <c r="AF684" t="inlineStr"/>
+      <c r="AG684" t="inlineStr"/>
+      <c r="AH684" t="inlineStr"/>
+      <c r="AI684" t="inlineStr"/>
+      <c r="AJ684" t="inlineStr">
+        <is>
+          <t>cl:10693</t>
+        </is>
+      </c>
+      <c r="AK684" t="inlineStr"/>
+      <c r="AL684" t="inlineStr"/>
+      <c r="AM684" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN684" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO684" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP684" t="inlineStr"/>
+      <c r="AQ684" t="inlineStr"/>
+      <c r="AR684" t="inlineStr"/>
+      <c r="AS684" t="inlineStr"/>
+      <c r="AT684" t="inlineStr"/>
+      <c r="AU684" t="inlineStr"/>
+      <c r="AV684" t="inlineStr"/>
+      <c r="AW684" t="inlineStr"/>
+      <c r="AX684" t="inlineStr"/>
+      <c r="AY684" t="inlineStr"/>
+      <c r="AZ684" t="inlineStr"/>
+      <c r="BA684" t="inlineStr"/>
+      <c r="BB684" t="inlineStr"/>
+      <c r="BC684" t="inlineStr"/>
+      <c r="BD684" t="inlineStr"/>
+      <c r="BE684" t="inlineStr"/>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>cl:10762</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Inland surface standing waters</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr"/>
+      <c r="F685" t="inlineStr"/>
+      <c r="G685" t="inlineStr"/>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>cl:10759</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr"/>
+      <c r="J685" t="inlineStr"/>
+      <c r="K685" t="inlineStr"/>
+      <c r="L685" t="inlineStr"/>
+      <c r="M685" t="inlineStr">
+        <is>
+          <t>cl:10651</t>
+        </is>
+      </c>
+      <c r="N685" t="inlineStr"/>
+      <c r="O685" t="inlineStr"/>
+      <c r="P685" t="inlineStr"/>
+      <c r="Q685" t="inlineStr"/>
+      <c r="R685" t="inlineStr"/>
+      <c r="S685" t="inlineStr"/>
+      <c r="T685" t="inlineStr"/>
+      <c r="U685" t="inlineStr"/>
+      <c r="V685" t="inlineStr"/>
+      <c r="W685" t="inlineStr"/>
+      <c r="X685" t="inlineStr"/>
+      <c r="Y685" t="inlineStr"/>
+      <c r="Z685" t="inlineStr"/>
+      <c r="AA685" t="inlineStr"/>
+      <c r="AB685" t="inlineStr"/>
+      <c r="AC685" t="inlineStr"/>
+      <c r="AD685" t="inlineStr"/>
+      <c r="AE685" t="inlineStr"/>
+      <c r="AF685" t="inlineStr"/>
+      <c r="AG685" t="inlineStr"/>
+      <c r="AH685" t="inlineStr"/>
+      <c r="AI685" t="inlineStr"/>
+      <c r="AJ685" t="inlineStr"/>
+      <c r="AK685" t="inlineStr"/>
+      <c r="AL685" t="inlineStr"/>
+      <c r="AM685" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN685" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO685" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP685" t="inlineStr"/>
+      <c r="AQ685" t="inlineStr"/>
+      <c r="AR685" t="inlineStr"/>
+      <c r="AS685" t="inlineStr"/>
+      <c r="AT685" t="inlineStr"/>
+      <c r="AU685" t="inlineStr"/>
+      <c r="AV685" t="inlineStr"/>
+      <c r="AW685" t="inlineStr"/>
+      <c r="AX685" t="inlineStr"/>
+      <c r="AY685" t="inlineStr"/>
+      <c r="AZ685" t="inlineStr"/>
+      <c r="BA685" t="inlineStr"/>
+      <c r="BB685" t="inlineStr"/>
+      <c r="BC685" t="inlineStr"/>
+      <c r="BD685" t="inlineStr"/>
+      <c r="BE685" t="inlineStr"/>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>cl:10763</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Inland surface running waters</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr"/>
+      <c r="F686" t="inlineStr"/>
+      <c r="G686" t="inlineStr"/>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>cl:10759</t>
+        </is>
+      </c>
+      <c r="I686" t="inlineStr"/>
+      <c r="J686" t="inlineStr"/>
+      <c r="K686" t="inlineStr"/>
+      <c r="L686" t="inlineStr"/>
+      <c r="M686" t="inlineStr">
+        <is>
+          <t>cl:10651</t>
+        </is>
+      </c>
+      <c r="N686" t="inlineStr"/>
+      <c r="O686" t="inlineStr"/>
+      <c r="P686" t="inlineStr"/>
+      <c r="Q686" t="inlineStr"/>
+      <c r="R686" t="inlineStr"/>
+      <c r="S686" t="inlineStr"/>
+      <c r="T686" t="inlineStr"/>
+      <c r="U686" t="inlineStr"/>
+      <c r="V686" t="inlineStr"/>
+      <c r="W686" t="inlineStr"/>
+      <c r="X686" t="inlineStr"/>
+      <c r="Y686" t="inlineStr"/>
+      <c r="Z686" t="inlineStr"/>
+      <c r="AA686" t="inlineStr"/>
+      <c r="AB686" t="inlineStr"/>
+      <c r="AC686" t="inlineStr"/>
+      <c r="AD686" t="inlineStr"/>
+      <c r="AE686" t="inlineStr"/>
+      <c r="AF686" t="inlineStr"/>
+      <c r="AG686" t="inlineStr"/>
+      <c r="AH686" t="inlineStr"/>
+      <c r="AI686" t="inlineStr"/>
+      <c r="AJ686" t="inlineStr"/>
+      <c r="AK686" t="inlineStr"/>
+      <c r="AL686" t="inlineStr"/>
+      <c r="AM686" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN686" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO686" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP686" t="inlineStr"/>
+      <c r="AQ686" t="inlineStr"/>
+      <c r="AR686" t="inlineStr"/>
+      <c r="AS686" t="inlineStr"/>
+      <c r="AT686" t="inlineStr"/>
+      <c r="AU686" t="inlineStr"/>
+      <c r="AV686" t="inlineStr"/>
+      <c r="AW686" t="inlineStr"/>
+      <c r="AX686" t="inlineStr"/>
+      <c r="AY686" t="inlineStr"/>
+      <c r="AZ686" t="inlineStr"/>
+      <c r="BA686" t="inlineStr"/>
+      <c r="BB686" t="inlineStr"/>
+      <c r="BC686" t="inlineStr"/>
+      <c r="BD686" t="inlineStr"/>
+      <c r="BE686" t="inlineStr"/>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>cl:10764</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Wetlands (mires, bogs, fens)</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr"/>
+      <c r="F687" t="inlineStr"/>
+      <c r="G687" t="inlineStr"/>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>cl:10759</t>
+        </is>
+      </c>
+      <c r="I687" t="inlineStr"/>
+      <c r="J687" t="inlineStr"/>
+      <c r="K687" t="inlineStr"/>
+      <c r="L687" t="inlineStr"/>
+      <c r="M687" t="inlineStr"/>
+      <c r="N687" t="inlineStr"/>
+      <c r="O687" t="inlineStr"/>
+      <c r="P687" t="inlineStr"/>
+      <c r="Q687" t="inlineStr"/>
+      <c r="R687" t="inlineStr"/>
+      <c r="S687" t="inlineStr"/>
+      <c r="T687" t="inlineStr"/>
+      <c r="U687" t="inlineStr"/>
+      <c r="V687" t="inlineStr"/>
+      <c r="W687" t="inlineStr"/>
+      <c r="X687" t="inlineStr"/>
+      <c r="Y687" t="inlineStr"/>
+      <c r="Z687" t="inlineStr"/>
+      <c r="AA687" t="inlineStr"/>
+      <c r="AB687" t="inlineStr"/>
+      <c r="AC687" t="inlineStr"/>
+      <c r="AD687" t="inlineStr"/>
+      <c r="AE687" t="inlineStr"/>
+      <c r="AF687" t="inlineStr"/>
+      <c r="AG687" t="inlineStr"/>
+      <c r="AH687" t="inlineStr"/>
+      <c r="AI687" t="inlineStr"/>
+      <c r="AJ687" t="inlineStr">
+        <is>
+          <t>cl:10652</t>
+        </is>
+      </c>
+      <c r="AK687" t="inlineStr"/>
+      <c r="AL687" t="inlineStr"/>
+      <c r="AM687" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN687" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO687" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP687" t="inlineStr"/>
+      <c r="AQ687" t="inlineStr"/>
+      <c r="AR687" t="inlineStr"/>
+      <c r="AS687" t="inlineStr"/>
+      <c r="AT687" t="inlineStr"/>
+      <c r="AU687" t="inlineStr"/>
+      <c r="AV687" t="inlineStr"/>
+      <c r="AW687" t="inlineStr"/>
+      <c r="AX687" t="inlineStr"/>
+      <c r="AY687" t="inlineStr"/>
+      <c r="AZ687" t="inlineStr"/>
+      <c r="BA687" t="inlineStr"/>
+      <c r="BB687" t="inlineStr"/>
+      <c r="BC687" t="inlineStr"/>
+      <c r="BD687" t="inlineStr"/>
+      <c r="BE687" t="inlineStr"/>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>cl:10765</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Grasslands and lands dominated by forbs, mosses or lichens</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr"/>
+      <c r="F688" t="inlineStr"/>
+      <c r="G688" t="inlineStr"/>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>cl:10759</t>
+        </is>
+      </c>
+      <c r="I688" t="inlineStr"/>
+      <c r="J688" t="inlineStr"/>
+      <c r="K688" t="inlineStr"/>
+      <c r="L688" t="inlineStr"/>
+      <c r="M688" t="inlineStr"/>
+      <c r="N688" t="inlineStr"/>
+      <c r="O688" t="inlineStr"/>
+      <c r="P688" t="inlineStr"/>
+      <c r="Q688" t="inlineStr"/>
+      <c r="R688" t="inlineStr"/>
+      <c r="S688" t="inlineStr"/>
+      <c r="T688" t="inlineStr"/>
+      <c r="U688" t="inlineStr"/>
+      <c r="V688" t="inlineStr"/>
+      <c r="W688" t="inlineStr"/>
+      <c r="X688" t="inlineStr"/>
+      <c r="Y688" t="inlineStr"/>
+      <c r="Z688" t="inlineStr"/>
+      <c r="AA688" t="inlineStr"/>
+      <c r="AB688" t="inlineStr"/>
+      <c r="AC688" t="inlineStr"/>
+      <c r="AD688" t="inlineStr"/>
+      <c r="AE688" t="inlineStr"/>
+      <c r="AF688" t="inlineStr"/>
+      <c r="AG688" t="inlineStr"/>
+      <c r="AH688" t="inlineStr"/>
+      <c r="AI688" t="inlineStr"/>
+      <c r="AJ688" t="inlineStr">
+        <is>
+          <t>cl:10653</t>
+        </is>
+      </c>
+      <c r="AK688" t="inlineStr"/>
+      <c r="AL688" t="inlineStr"/>
+      <c r="AM688" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN688" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO688" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP688" t="inlineStr"/>
+      <c r="AQ688" t="inlineStr"/>
+      <c r="AR688" t="inlineStr"/>
+      <c r="AS688" t="inlineStr"/>
+      <c r="AT688" t="inlineStr"/>
+      <c r="AU688" t="inlineStr"/>
+      <c r="AV688" t="inlineStr"/>
+      <c r="AW688" t="inlineStr"/>
+      <c r="AX688" t="inlineStr"/>
+      <c r="AY688" t="inlineStr"/>
+      <c r="AZ688" t="inlineStr"/>
+      <c r="BA688" t="inlineStr"/>
+      <c r="BB688" t="inlineStr"/>
+      <c r="BC688" t="inlineStr"/>
+      <c r="BD688" t="inlineStr"/>
+      <c r="BE688" t="inlineStr"/>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>cl:10766</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Heathlands, shrub and tundra</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr"/>
+      <c r="F689" t="inlineStr"/>
+      <c r="G689" t="inlineStr"/>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>cl:10759</t>
+        </is>
+      </c>
+      <c r="I689" t="inlineStr"/>
+      <c r="J689" t="inlineStr"/>
+      <c r="K689" t="inlineStr"/>
+      <c r="L689" t="inlineStr"/>
+      <c r="M689" t="inlineStr"/>
+      <c r="N689" t="inlineStr"/>
+      <c r="O689" t="inlineStr"/>
+      <c r="P689" t="inlineStr"/>
+      <c r="Q689" t="inlineStr"/>
+      <c r="R689" t="inlineStr"/>
+      <c r="S689" t="inlineStr"/>
+      <c r="T689" t="inlineStr"/>
+      <c r="U689" t="inlineStr"/>
+      <c r="V689" t="inlineStr"/>
+      <c r="W689" t="inlineStr"/>
+      <c r="X689" t="inlineStr"/>
+      <c r="Y689" t="inlineStr"/>
+      <c r="Z689" t="inlineStr"/>
+      <c r="AA689" t="inlineStr"/>
+      <c r="AB689" t="inlineStr"/>
+      <c r="AC689" t="inlineStr"/>
+      <c r="AD689" t="inlineStr"/>
+      <c r="AE689" t="inlineStr"/>
+      <c r="AF689" t="inlineStr"/>
+      <c r="AG689" t="inlineStr"/>
+      <c r="AH689" t="inlineStr"/>
+      <c r="AI689" t="inlineStr"/>
+      <c r="AJ689" t="inlineStr">
+        <is>
+          <t>cl:10654</t>
+        </is>
+      </c>
+      <c r="AK689" t="inlineStr"/>
+      <c r="AL689" t="inlineStr"/>
+      <c r="AM689" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN689" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO689" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP689" t="inlineStr"/>
+      <c r="AQ689" t="inlineStr"/>
+      <c r="AR689" t="inlineStr"/>
+      <c r="AS689" t="inlineStr"/>
+      <c r="AT689" t="inlineStr"/>
+      <c r="AU689" t="inlineStr"/>
+      <c r="AV689" t="inlineStr"/>
+      <c r="AW689" t="inlineStr"/>
+      <c r="AX689" t="inlineStr"/>
+      <c r="AY689" t="inlineStr"/>
+      <c r="AZ689" t="inlineStr"/>
+      <c r="BA689" t="inlineStr"/>
+      <c r="BB689" t="inlineStr"/>
+      <c r="BC689" t="inlineStr"/>
+      <c r="BD689" t="inlineStr"/>
+      <c r="BE689" t="inlineStr"/>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>cl:10767</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Forests and other wooded land</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr"/>
+      <c r="F690" t="inlineStr"/>
+      <c r="G690" t="inlineStr"/>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>cl:10759</t>
+        </is>
+      </c>
+      <c r="I690" t="inlineStr"/>
+      <c r="J690" t="inlineStr"/>
+      <c r="K690" t="inlineStr"/>
+      <c r="L690" t="inlineStr"/>
+      <c r="M690" t="inlineStr"/>
+      <c r="N690" t="inlineStr"/>
+      <c r="O690" t="inlineStr"/>
+      <c r="P690" t="inlineStr"/>
+      <c r="Q690" t="inlineStr"/>
+      <c r="R690" t="inlineStr"/>
+      <c r="S690" t="inlineStr"/>
+      <c r="T690" t="inlineStr"/>
+      <c r="U690" t="inlineStr"/>
+      <c r="V690" t="inlineStr"/>
+      <c r="W690" t="inlineStr"/>
+      <c r="X690" t="inlineStr"/>
+      <c r="Y690" t="inlineStr"/>
+      <c r="Z690" t="inlineStr"/>
+      <c r="AA690" t="inlineStr"/>
+      <c r="AB690" t="inlineStr"/>
+      <c r="AC690" t="inlineStr"/>
+      <c r="AD690" t="inlineStr"/>
+      <c r="AE690" t="inlineStr"/>
+      <c r="AF690" t="inlineStr"/>
+      <c r="AG690" t="inlineStr"/>
+      <c r="AH690" t="inlineStr"/>
+      <c r="AI690" t="inlineStr"/>
+      <c r="AJ690" t="inlineStr">
+        <is>
+          <t>cl:10655</t>
+        </is>
+      </c>
+      <c r="AK690" t="inlineStr"/>
+      <c r="AL690" t="inlineStr"/>
+      <c r="AM690" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN690" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO690" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP690" t="inlineStr"/>
+      <c r="AQ690" t="inlineStr"/>
+      <c r="AR690" t="inlineStr"/>
+      <c r="AS690" t="inlineStr"/>
+      <c r="AT690" t="inlineStr"/>
+      <c r="AU690" t="inlineStr"/>
+      <c r="AV690" t="inlineStr"/>
+      <c r="AW690" t="inlineStr"/>
+      <c r="AX690" t="inlineStr"/>
+      <c r="AY690" t="inlineStr"/>
+      <c r="AZ690" t="inlineStr"/>
+      <c r="BA690" t="inlineStr"/>
+      <c r="BB690" t="inlineStr"/>
+      <c r="BC690" t="inlineStr"/>
+      <c r="BD690" t="inlineStr"/>
+      <c r="BE690" t="inlineStr"/>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>cl:10768</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Sparsely vegetated habitats and deserts</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr"/>
+      <c r="F691" t="inlineStr"/>
+      <c r="G691" t="inlineStr"/>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>cl:10759</t>
+        </is>
+      </c>
+      <c r="I691" t="inlineStr"/>
+      <c r="J691" t="inlineStr"/>
+      <c r="K691" t="inlineStr"/>
+      <c r="L691" t="inlineStr"/>
+      <c r="M691" t="inlineStr"/>
+      <c r="N691" t="inlineStr"/>
+      <c r="O691" t="inlineStr"/>
+      <c r="P691" t="inlineStr"/>
+      <c r="Q691" t="inlineStr"/>
+      <c r="R691" t="inlineStr"/>
+      <c r="S691" t="inlineStr"/>
+      <c r="T691" t="inlineStr"/>
+      <c r="U691" t="inlineStr"/>
+      <c r="V691" t="inlineStr"/>
+      <c r="W691" t="inlineStr"/>
+      <c r="X691" t="inlineStr"/>
+      <c r="Y691" t="inlineStr"/>
+      <c r="Z691" t="inlineStr"/>
+      <c r="AA691" t="inlineStr"/>
+      <c r="AB691" t="inlineStr"/>
+      <c r="AC691" t="inlineStr"/>
+      <c r="AD691" t="inlineStr"/>
+      <c r="AE691" t="inlineStr"/>
+      <c r="AF691" t="inlineStr"/>
+      <c r="AG691" t="inlineStr"/>
+      <c r="AH691" t="inlineStr"/>
+      <c r="AI691" t="inlineStr"/>
+      <c r="AJ691" t="inlineStr">
+        <is>
+          <t>cl:10656</t>
+        </is>
+      </c>
+      <c r="AK691" t="inlineStr"/>
+      <c r="AL691" t="inlineStr"/>
+      <c r="AM691" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN691" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO691" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP691" t="inlineStr"/>
+      <c r="AQ691" t="inlineStr"/>
+      <c r="AR691" t="inlineStr"/>
+      <c r="AS691" t="inlineStr"/>
+      <c r="AT691" t="inlineStr"/>
+      <c r="AU691" t="inlineStr"/>
+      <c r="AV691" t="inlineStr"/>
+      <c r="AW691" t="inlineStr"/>
+      <c r="AX691" t="inlineStr"/>
+      <c r="AY691" t="inlineStr"/>
+      <c r="AZ691" t="inlineStr"/>
+      <c r="BA691" t="inlineStr"/>
+      <c r="BB691" t="inlineStr"/>
+      <c r="BC691" t="inlineStr"/>
+      <c r="BD691" t="inlineStr"/>
+      <c r="BE691" t="inlineStr"/>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>cl:10769</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Vegetated man-made habitats (agricultural, horticultural, domestic)</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>skos:Concept</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr"/>
+      <c r="F692" t="inlineStr"/>
+      <c r="G692" t="inlineStr"/>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>cl:10759</t>
+        </is>
+      </c>
+      <c r="I692" t="inlineStr"/>
+      <c r="J692" t="inlineStr"/>
+      <c r="K692" t="inlineStr"/>
+      <c r="L692" t="inlineStr"/>
+      <c r="M692" t="inlineStr"/>
+      <c r="N692" t="inlineStr"/>
+      <c r="O692" t="inlineStr"/>
+      <c r="P692" t="inlineStr"/>
+      <c r="Q692" t="inlineStr"/>
+      <c r="R692" t="inlineStr"/>
+      <c r="S692" t="inlineStr"/>
+      <c r="T692" t="inlineStr"/>
+      <c r="U692" t="inlineStr"/>
+      <c r="V692" t="inlineStr"/>
+      <c r="W692" t="inlineStr"/>
+      <c r="X692" t="inlineStr"/>
+      <c r="Y692" t="inlineStr"/>
+      <c r="Z692" t="inlineStr"/>
+      <c r="AA692" t="inlineStr"/>
+      <c r="AB692" t="inlineStr"/>
+      <c r="AC692" t="inlineStr"/>
+      <c r="AD692" t="inlineStr"/>
+      <c r="AE692" t="inlineStr"/>
+      <c r="AF692" t="inlineStr"/>
+      <c r="AG692" t="inlineStr"/>
+      <c r="AH692" t="inlineStr"/>
+      <c r="AI692" t="inlineStr"/>
+      <c r="AJ692" t="inlineStr">
+        <is>
+          <t>cl:10657</t>
+        </is>
+      </c>
+      <c r="AK692" t="inlineStr"/>
+      <c r="AL692" t="inlineStr"/>
+      <c r="AM692" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AN692" t="inlineStr">
+        <is>
+          <t>0000-0002-7997-219X</t>
+        </is>
+      </c>
+      <c r="AO692" t="inlineStr">
+        <is>
+          <t>11/26/2025</t>
+        </is>
+      </c>
+      <c r="AP692" t="inlineStr"/>
+      <c r="AQ692" t="inlineStr"/>
+      <c r="AR692" t="inlineStr"/>
+      <c r="AS692" t="inlineStr"/>
+      <c r="AT692" t="inlineStr"/>
+      <c r="AU692" t="inlineStr"/>
+      <c r="AV692" t="inlineStr"/>
+      <c r="AW692" t="inlineStr"/>
+      <c r="AX692" t="inlineStr"/>
+      <c r="AY692" t="inlineStr"/>
+      <c r="AZ692" t="inlineStr"/>
+      <c r="BA692" t="inlineStr"/>
+      <c r="BB692" t="inlineStr"/>
+      <c r="BC692" t="inlineStr"/>
+      <c r="BD692" t="inlineStr"/>
+      <c r="BE692" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>